<commit_message>
logic function - hanging flowchart
</commit_message>
<xml_diff>
--- a/1.training_model/supplementary/Data Tabulation - Flowchart.xlsx
+++ b/1.training_model/supplementary/Data Tabulation - Flowchart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sitisyaziyah\source\repos\DeviceCluster\1.training_model\supplementary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAD0E266-0574-4133-946C-BC5074C83765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A10780F-3F7D-46DD-A140-9ABCD75F2469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="717" activeTab="5" xr2:uid="{E471D6E3-533D-4285-ABDC-6FF3DFDEE99D}"/>
   </bookViews>
@@ -17,17 +17,17 @@
     <sheet name="Stage 1" sheetId="4" r:id="rId2"/>
     <sheet name="Stage 2" sheetId="6" r:id="rId3"/>
     <sheet name="Stage 3" sheetId="7" r:id="rId4"/>
-    <sheet name="Stage 4" sheetId="8" r:id="rId5"/>
-    <sheet name="Stage 4 (2)" sheetId="13" r:id="rId6"/>
+    <sheet name="Stage 4" sheetId="13" r:id="rId5"/>
+    <sheet name="draft" sheetId="15" r:id="rId6"/>
     <sheet name="Example case" sheetId="12" r:id="rId7"/>
     <sheet name="transpose" sheetId="3" state="hidden" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Stage 1'!$B$2:$H$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">draft!#REF!</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Stage 1'!$B$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stage 2'!$B$2:$H$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Stage 3'!$B$2:$H$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Stage 4'!#REF!</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Stage 4 (2)'!#REF!</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">transpose!$B$3:$AE$12</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="67">
   <si>
     <t>Device ID</t>
   </si>
@@ -241,12 +241,24 @@
   <si>
     <t>Catagorize Device ID by each  cluster group</t>
   </si>
+  <si>
+    <t>Sort the highest percentage for each cluster</t>
+  </si>
+  <si>
+    <t>VACANT</t>
+  </si>
+  <si>
+    <t>Control Valve</t>
+  </si>
+  <si>
+    <t>Check the vacant and extra</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -270,8 +282,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -311,6 +331,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -355,10 +381,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -399,8 +426,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -421,15 +464,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>499242</xdr:colOff>
+      <xdr:colOff>485589</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>123519</xdr:rowOff>
+      <xdr:rowOff>140157</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>160338</xdr:colOff>
+      <xdr:colOff>146685</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>101929</xdr:rowOff>
+      <xdr:rowOff>118567</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -444,8 +487,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6746328" y="1411036"/>
-          <a:ext cx="2104751" cy="543341"/>
+          <a:off x="6722276" y="1412401"/>
+          <a:ext cx="2097881" cy="543852"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -498,15 +541,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>160338</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>168808</xdr:rowOff>
+      <xdr:colOff>143510</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>33060</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>371346</xdr:colOff>
+      <xdr:colOff>354708</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>20759</xdr:rowOff>
+      <xdr:rowOff>41663</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -524,8 +567,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="8851079" y="1640256"/>
-          <a:ext cx="2654664" cy="42451"/>
+          <a:off x="8816982" y="1678899"/>
+          <a:ext cx="2647982" cy="8603"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -554,15 +597,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>374521</xdr:colOff>
+      <xdr:colOff>357883</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>48816</xdr:rowOff>
+      <xdr:rowOff>99301</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
-      <xdr:colOff>579674</xdr:colOff>
+      <xdr:colOff>569386</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>94906</xdr:rowOff>
+      <xdr:rowOff>142216</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -577,8 +620,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11490196" y="1315641"/>
-          <a:ext cx="2033953" cy="608065"/>
+          <a:off x="11468139" y="1371545"/>
+          <a:ext cx="2039092" cy="608357"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -635,15 +678,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>329790</xdr:colOff>
+      <xdr:colOff>316137</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>45641</xdr:rowOff>
+      <xdr:rowOff>102476</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>171641</xdr:colOff>
+      <xdr:colOff>157450</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>123519</xdr:rowOff>
+      <xdr:rowOff>143332</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -661,12 +704,12 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm rot="16200000" flipH="1" flipV="1">
-          <a:off x="10124346" y="-992484"/>
-          <a:ext cx="77878" cy="4729161"/>
+          <a:off x="10108230" y="-962293"/>
+          <a:ext cx="40856" cy="4714881"/>
         </a:xfrm>
         <a:prstGeom prst="bentConnector3">
           <a:avLst>
-            <a:gd name="adj1" fmla="val -293536"/>
+            <a:gd name="adj1" fmla="val -559526"/>
           </a:avLst>
         </a:prstGeom>
         <a:ln>
@@ -829,15 +872,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>245012</xdr:colOff>
+      <xdr:colOff>216640</xdr:colOff>
       <xdr:row>13</xdr:row>
-      <xdr:rowOff>168820</xdr:rowOff>
+      <xdr:rowOff>164766</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>406937</xdr:colOff>
+      <xdr:colOff>381740</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>112995</xdr:rowOff>
+      <xdr:rowOff>108941</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -852,8 +895,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6492098" y="2573061"/>
-          <a:ext cx="2605580" cy="312037"/>
+          <a:off x="6450449" y="2552096"/>
+          <a:ext cx="2597014" cy="308962"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -906,15 +949,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>327562</xdr:colOff>
+      <xdr:colOff>300778</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>105104</xdr:rowOff>
+      <xdr:rowOff>121742</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>332965</xdr:colOff>
+      <xdr:colOff>316137</xdr:colOff>
       <xdr:row>13</xdr:row>
-      <xdr:rowOff>168820</xdr:rowOff>
+      <xdr:rowOff>161591</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -932,8 +975,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="7796476" y="1957552"/>
-          <a:ext cx="5403" cy="615509"/>
+          <a:off x="7750544" y="1961891"/>
+          <a:ext cx="15359" cy="587030"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -1020,9 +1063,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>576384</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>107462</xdr:rowOff>
+      <xdr:colOff>587666</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>156978</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="346826" cy="264560"/>
     <xdr:sp macro="" textlink="">
@@ -1038,7 +1081,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6530730" y="1973385"/>
+          <a:off x="7429453" y="2179521"/>
           <a:ext cx="346826" cy="264560"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1078,15 +1121,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>245672</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>24221</xdr:rowOff>
+      <xdr:colOff>213246</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>153045</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>416981</xdr:colOff>
+      <xdr:colOff>384555</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>107046</xdr:rowOff>
+      <xdr:rowOff>47126</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1101,8 +1144,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6492758" y="3348118"/>
-          <a:ext cx="2614964" cy="450687"/>
+          <a:off x="6447055" y="3269949"/>
+          <a:ext cx="2603223" cy="441262"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1155,15 +1198,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>327562</xdr:colOff>
+      <xdr:colOff>300778</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>112995</xdr:rowOff>
+      <xdr:rowOff>105766</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>331326</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>27396</xdr:rowOff>
+      <xdr:colOff>302076</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>153045</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -1181,8 +1224,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7796476" y="2885098"/>
-          <a:ext cx="3764" cy="466195"/>
+          <a:off x="7750544" y="2857883"/>
+          <a:ext cx="1298" cy="412066"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -1211,15 +1254,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>160338</xdr:colOff>
+      <xdr:colOff>146685</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>20759</xdr:rowOff>
+      <xdr:rowOff>34222</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>207031</xdr:colOff>
+      <xdr:colOff>190203</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>114848</xdr:rowOff>
+      <xdr:rowOff>128311</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -1236,8 +1279,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8851079" y="1682707"/>
-          <a:ext cx="2490349" cy="1388175"/>
+          <a:off x="8820157" y="1680061"/>
+          <a:ext cx="2480302" cy="1376430"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -1780,7 +1823,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EFAC392-3DBC-4888-8676-CE4E321B2BF1}">
-  <dimension ref="B2:Q31"/>
+  <dimension ref="B1:Q30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="9.08984375" bestFit="1" customWidth="1"/>
@@ -1794,74 +1837,112 @@
     <col min="13" max="13" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="B1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="L1" t="s">
+        <v>39</v>
+      </c>
+      <c r="M1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N1" t="s">
+        <v>40</v>
+      </c>
+      <c r="O1" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
     <row r="2" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B2" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="10" t="s">
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2">
+        <v>68.8</v>
+      </c>
+      <c r="E2">
+        <v>83.4</v>
+      </c>
+      <c r="F2">
+        <v>19.8</v>
+      </c>
+      <c r="G2">
+        <v>38.200000000000003</v>
+      </c>
+      <c r="H2" s="4">
+        <v>84</v>
+      </c>
+      <c r="K2" t="s">
+        <v>42</v>
+      </c>
+      <c r="L2">
+        <v>2</v>
+      </c>
+      <c r="M2">
         <v>1</v>
       </c>
-      <c r="D2" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="10" t="s">
+      <c r="N2">
         <v>3</v>
       </c>
-      <c r="F2" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="G2" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" s="10" t="s">
+      <c r="O2" s="12">
         <v>6</v>
-      </c>
-      <c r="L2" t="s">
-        <v>39</v>
-      </c>
-      <c r="M2" t="s">
-        <v>41</v>
-      </c>
-      <c r="N2" t="s">
-        <v>40</v>
-      </c>
-      <c r="O2" s="12" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="3" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
         <v>8</v>
       </c>
       <c r="D3">
-        <v>68.8</v>
+        <v>69.2</v>
       </c>
       <c r="E3">
-        <v>83.4</v>
-      </c>
-      <c r="F3">
-        <v>19.8</v>
+        <v>83</v>
+      </c>
+      <c r="F3" s="4">
+        <v>91</v>
       </c>
       <c r="G3">
-        <v>38.200000000000003</v>
-      </c>
-      <c r="H3" s="4">
-        <v>84</v>
+        <v>56.2</v>
+      </c>
+      <c r="H3">
+        <v>79.8</v>
       </c>
       <c r="K3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L3">
         <v>2</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O3" s="12">
         <v>6</v>
@@ -1869,760 +1950,722 @@
     </row>
     <row r="4" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
         <v>8</v>
       </c>
       <c r="D4">
-        <v>69.2</v>
+        <v>19.8</v>
       </c>
       <c r="E4">
-        <v>83</v>
+        <v>33.200000000000003</v>
       </c>
       <c r="F4" s="4">
-        <v>91</v>
+        <v>95.3</v>
       </c>
       <c r="G4">
-        <v>56.2</v>
+        <v>12.4</v>
       </c>
       <c r="H4">
-        <v>79.8</v>
+        <v>57.9</v>
       </c>
       <c r="K4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O4" s="12">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
         <v>8</v>
       </c>
-      <c r="D5">
-        <v>19.8</v>
+      <c r="D5" s="4">
+        <v>98.5</v>
       </c>
       <c r="E5">
-        <v>33.200000000000003</v>
-      </c>
-      <c r="F5" s="4">
-        <v>95.3</v>
+        <v>84.4</v>
+      </c>
+      <c r="F5">
+        <v>7.2</v>
       </c>
       <c r="G5">
-        <v>12.4</v>
+        <v>83</v>
       </c>
       <c r="H5">
-        <v>57.9</v>
+        <v>31.2</v>
       </c>
       <c r="K5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M5">
         <v>1</v>
       </c>
       <c r="N5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O5" s="12">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="4">
-        <v>98.5</v>
+      <c r="D6">
+        <v>39.6</v>
       </c>
       <c r="E6">
-        <v>84.4</v>
+        <v>1.3</v>
       </c>
       <c r="F6">
-        <v>7.2</v>
+        <v>54.9</v>
       </c>
       <c r="G6">
-        <v>83</v>
-      </c>
-      <c r="H6">
-        <v>31.2</v>
+        <v>26.3</v>
+      </c>
+      <c r="H6" s="4">
+        <v>65</v>
       </c>
       <c r="K6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O6" s="12">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C7" t="s">
         <v>8</v>
       </c>
       <c r="D7">
-        <v>39.6</v>
-      </c>
-      <c r="E7">
-        <v>1.3</v>
+        <v>67.900000000000006</v>
+      </c>
+      <c r="E7" s="4">
+        <v>84.7</v>
       </c>
       <c r="F7">
-        <v>54.9</v>
+        <v>35.700000000000003</v>
       </c>
       <c r="G7">
-        <v>26.3</v>
-      </c>
-      <c r="H7" s="4">
-        <v>65</v>
-      </c>
-      <c r="K7" t="s">
-        <v>46</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
-        <v>0</v>
-      </c>
-      <c r="N7">
+        <v>21.3</v>
+      </c>
+      <c r="H7">
+        <v>43.2</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="L7" s="11">
+        <v>10</v>
+      </c>
+      <c r="M7" s="11">
         <v>5</v>
       </c>
-      <c r="O7" s="12">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="N7" s="11">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="2:17" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C8" t="s">
         <v>8</v>
       </c>
       <c r="D8">
-        <v>67.900000000000006</v>
-      </c>
-      <c r="E8" s="4">
-        <v>84.7</v>
+        <v>44.5</v>
+      </c>
+      <c r="E8">
+        <v>16.8</v>
       </c>
       <c r="F8">
-        <v>35.700000000000003</v>
-      </c>
-      <c r="G8">
-        <v>21.3</v>
+        <v>73.099999999999994</v>
+      </c>
+      <c r="G8" s="4">
+        <v>76.400000000000006</v>
       </c>
       <c r="H8">
-        <v>43.2</v>
-      </c>
-      <c r="K8" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="L8" s="11">
-        <v>10</v>
-      </c>
-      <c r="M8" s="11">
-        <v>5</v>
-      </c>
-      <c r="N8" s="11">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="2:17" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+        <v>8.6</v>
+      </c>
+    </row>
+    <row r="9" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s">
         <v>8</v>
       </c>
       <c r="D9">
-        <v>44.5</v>
+        <v>46.3</v>
       </c>
       <c r="E9">
-        <v>16.8</v>
-      </c>
-      <c r="F9">
-        <v>73.099999999999994</v>
-      </c>
-      <c r="G9" s="4">
-        <v>76.400000000000006</v>
+        <v>24.1</v>
+      </c>
+      <c r="F9" s="4">
+        <v>87.1</v>
+      </c>
+      <c r="G9">
+        <v>47.8</v>
       </c>
       <c r="H9">
-        <v>8.6</v>
+        <v>30.2</v>
       </c>
     </row>
     <row r="10" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C10" t="s">
         <v>8</v>
       </c>
-      <c r="D10">
-        <v>46.3</v>
+      <c r="D10" s="4">
+        <v>96.8</v>
       </c>
       <c r="E10">
-        <v>24.1</v>
-      </c>
-      <c r="F10" s="4">
-        <v>87.1</v>
+        <v>64.900000000000006</v>
+      </c>
+      <c r="F10">
+        <v>7</v>
       </c>
       <c r="G10">
-        <v>47.8</v>
+        <v>78.8</v>
       </c>
       <c r="H10">
-        <v>30.2</v>
-      </c>
-    </row>
-    <row r="11" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" s="4">
-        <v>96.8</v>
-      </c>
-      <c r="E11">
-        <v>64.900000000000006</v>
-      </c>
-      <c r="F11">
-        <v>7</v>
-      </c>
-      <c r="G11">
-        <v>78.8</v>
-      </c>
-      <c r="H11">
         <v>22.2</v>
       </c>
-      <c r="K11" s="13" t="s">
+      <c r="K10" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="L11" s="13" t="s">
+      <c r="L10" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="M11" s="13"/>
-      <c r="N11" s="13"/>
-      <c r="O11" s="13"/>
-      <c r="P11" s="1"/>
-      <c r="Q11" s="1"/>
-    </row>
-    <row r="12" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="9" t="s">
+      <c r="M10" s="13"/>
+      <c r="N10" s="13"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="1"/>
+      <c r="Q10" s="1"/>
+    </row>
+    <row r="11" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B11" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" s="9">
+      <c r="C11" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="9">
         <v>78.900000000000006</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E11" s="9">
         <v>84</v>
       </c>
-      <c r="F12" s="9">
+      <c r="F11" s="9">
         <v>22.4</v>
       </c>
-      <c r="G12" s="17">
+      <c r="G11" s="17">
         <v>89.1</v>
       </c>
-      <c r="H12" s="9">
+      <c r="H11" s="9">
         <v>35.700000000000003</v>
       </c>
-      <c r="K12" t="s">
+      <c r="K11" t="s">
         <v>50</v>
       </c>
+      <c r="L11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12">
+        <v>50.9</v>
+      </c>
+      <c r="E12">
+        <v>46</v>
+      </c>
+      <c r="F12">
+        <v>7.2</v>
+      </c>
+      <c r="G12">
+        <v>7.4</v>
+      </c>
+      <c r="H12" s="4">
+        <v>90.3</v>
+      </c>
       <c r="L12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C13" t="s">
         <v>19</v>
       </c>
-      <c r="D13">
-        <v>50.9</v>
+      <c r="D13" s="4">
+        <v>76.7</v>
       </c>
       <c r="E13">
-        <v>46</v>
+        <v>52.8</v>
       </c>
       <c r="F13">
-        <v>7.2</v>
+        <v>1.3</v>
       </c>
       <c r="G13">
-        <v>7.4</v>
-      </c>
-      <c r="H13" s="4">
-        <v>90.3</v>
-      </c>
-      <c r="L13" t="s">
-        <v>52</v>
+        <v>0.7</v>
+      </c>
+      <c r="H13">
+        <v>19.7</v>
+      </c>
+      <c r="L13" s="18" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C14" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="4">
-        <v>76.7</v>
+      <c r="D14">
+        <v>28.3</v>
       </c>
       <c r="E14">
-        <v>52.8</v>
+        <v>40.4</v>
       </c>
       <c r="F14">
-        <v>1.3</v>
+        <v>12.6</v>
       </c>
       <c r="G14">
-        <v>0.7</v>
-      </c>
-      <c r="H14">
-        <v>19.7</v>
-      </c>
-      <c r="L14" s="18" t="s">
-        <v>55</v>
+        <v>43.9</v>
+      </c>
+      <c r="H14" s="4">
+        <v>84.7</v>
+      </c>
+      <c r="L14" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C15" t="s">
         <v>19</v>
       </c>
       <c r="D15">
-        <v>28.3</v>
+        <v>8.5</v>
       </c>
       <c r="E15">
-        <v>40.4</v>
+        <v>60.3</v>
       </c>
       <c r="F15">
-        <v>12.6</v>
+        <v>27.9</v>
       </c>
       <c r="G15">
-        <v>43.9</v>
+        <v>31.8</v>
       </c>
       <c r="H15" s="4">
-        <v>84.7</v>
+        <v>66.7</v>
+      </c>
+      <c r="K15" t="s">
+        <v>54</v>
       </c>
       <c r="L15" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B16" t="s">
-        <v>22</v>
-      </c>
-      <c r="C16" t="s">
+    <row r="16" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B16" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D16">
-        <v>8.5</v>
-      </c>
-      <c r="E16">
-        <v>60.3</v>
-      </c>
-      <c r="F16">
-        <v>27.9</v>
-      </c>
-      <c r="G16">
-        <v>31.8</v>
-      </c>
-      <c r="H16" s="4">
-        <v>66.7</v>
+      <c r="D16" s="9">
+        <v>14.3</v>
+      </c>
+      <c r="E16" s="9">
+        <v>45</v>
+      </c>
+      <c r="F16" s="17">
+        <v>73.3</v>
+      </c>
+      <c r="G16" s="9">
+        <v>51.8</v>
+      </c>
+      <c r="H16" s="9">
+        <v>36.1</v>
       </c>
       <c r="K16" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="L16" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="17" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B17" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D17" s="9">
-        <v>14.3</v>
-      </c>
-      <c r="E17" s="9">
-        <v>45</v>
-      </c>
-      <c r="F17" s="17">
-        <v>73.3</v>
-      </c>
-      <c r="G17" s="9">
-        <v>51.8</v>
-      </c>
-      <c r="H17" s="9">
-        <v>36.1</v>
-      </c>
-      <c r="K17" t="s">
-        <v>56</v>
-      </c>
-      <c r="L17" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B17" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17">
+        <v>47.4</v>
+      </c>
+      <c r="E17">
+        <v>72.5</v>
+      </c>
+      <c r="F17">
+        <v>74.900000000000006</v>
+      </c>
+      <c r="G17" s="4">
+        <v>84.3</v>
+      </c>
+      <c r="H17">
+        <v>18.899999999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C18" t="s">
         <v>25</v>
       </c>
       <c r="D18">
-        <v>47.4</v>
-      </c>
-      <c r="E18">
-        <v>72.5</v>
+        <v>58.9</v>
+      </c>
+      <c r="E18" s="4">
+        <v>99</v>
       </c>
       <c r="F18">
-        <v>74.900000000000006</v>
-      </c>
-      <c r="G18" s="4">
-        <v>84.3</v>
+        <v>92.4</v>
+      </c>
+      <c r="G18">
+        <v>57.6</v>
       </c>
       <c r="H18">
-        <v>18.899999999999999</v>
-      </c>
-    </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+        <v>89.7</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C19" t="s">
         <v>25</v>
       </c>
       <c r="D19">
-        <v>58.9</v>
-      </c>
-      <c r="E19" s="4">
-        <v>99</v>
-      </c>
-      <c r="F19">
-        <v>92.4</v>
+        <v>55.1</v>
+      </c>
+      <c r="E19">
+        <v>20.9</v>
+      </c>
+      <c r="F19" s="4">
+        <v>86</v>
       </c>
       <c r="G19">
-        <v>57.6</v>
+        <v>77.8</v>
       </c>
       <c r="H19">
-        <v>89.7</v>
-      </c>
-    </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+        <v>54.7</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C20" t="s">
         <v>25</v>
       </c>
       <c r="D20">
-        <v>55.1</v>
+        <v>16.3</v>
       </c>
       <c r="E20">
-        <v>20.9</v>
-      </c>
-      <c r="F20" s="4">
-        <v>86</v>
-      </c>
-      <c r="G20">
-        <v>77.8</v>
+        <v>22.8</v>
+      </c>
+      <c r="F20">
+        <v>82</v>
+      </c>
+      <c r="G20" s="4">
+        <v>96.9</v>
       </c>
       <c r="H20">
-        <v>54.7</v>
-      </c>
-    </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
+        <v>28.7</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B21" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C21" t="s">
         <v>25</v>
       </c>
-      <c r="D21">
-        <v>16.3</v>
+      <c r="D21" s="4">
+        <v>83.9</v>
       </c>
       <c r="E21">
-        <v>22.8</v>
+        <v>4.8</v>
       </c>
       <c r="F21">
-        <v>82</v>
-      </c>
-      <c r="G21" s="4">
-        <v>96.9</v>
+        <v>70.2</v>
+      </c>
+      <c r="G21">
+        <v>58.1</v>
       </c>
       <c r="H21">
-        <v>28.7</v>
-      </c>
-    </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+        <v>46.3</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C22" t="s">
         <v>25</v>
       </c>
       <c r="D22" s="4">
-        <v>83.9</v>
+        <v>70</v>
       </c>
       <c r="E22">
+        <v>5.9</v>
+      </c>
+      <c r="F22">
+        <v>26.7</v>
+      </c>
+      <c r="G22">
+        <v>18.399999999999999</v>
+      </c>
+      <c r="H22">
+        <v>41.7</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B23" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" t="s">
+        <v>25</v>
+      </c>
+      <c r="D23">
+        <v>52.5</v>
+      </c>
+      <c r="E23">
+        <v>71.5</v>
+      </c>
+      <c r="F23">
+        <v>7</v>
+      </c>
+      <c r="G23">
+        <v>70.3</v>
+      </c>
+      <c r="H23" s="4">
+        <v>91.7</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B24" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" t="s">
+        <v>25</v>
+      </c>
+      <c r="D24">
+        <v>3.4</v>
+      </c>
+      <c r="E24">
+        <v>63.3</v>
+      </c>
+      <c r="F24">
+        <v>36.200000000000003</v>
+      </c>
+      <c r="G24" s="4">
+        <v>70.5</v>
+      </c>
+      <c r="H24">
+        <v>63.8</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" t="s">
+        <v>25</v>
+      </c>
+      <c r="D25">
+        <v>57.9</v>
+      </c>
+      <c r="E25">
+        <v>50.4</v>
+      </c>
+      <c r="F25">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="G25" s="4">
+        <v>63.4</v>
+      </c>
+      <c r="H25">
         <v>4.8</v>
       </c>
-      <c r="F22">
-        <v>70.2</v>
-      </c>
-      <c r="G22">
-        <v>58.1</v>
-      </c>
-      <c r="H22">
-        <v>46.3</v>
-      </c>
-    </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B23" t="s">
-        <v>30</v>
-      </c>
-      <c r="C23" t="s">
-        <v>25</v>
-      </c>
-      <c r="D23" s="4">
-        <v>70</v>
-      </c>
-      <c r="E23">
-        <v>5.9</v>
-      </c>
-      <c r="F23">
-        <v>26.7</v>
-      </c>
-      <c r="G23">
-        <v>18.399999999999999</v>
-      </c>
-      <c r="H23">
-        <v>41.7</v>
-      </c>
-    </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B24" t="s">
-        <v>31</v>
-      </c>
-      <c r="C24" t="s">
-        <v>25</v>
-      </c>
-      <c r="D24">
-        <v>52.5</v>
-      </c>
-      <c r="E24">
-        <v>71.5</v>
-      </c>
-      <c r="F24">
-        <v>7</v>
-      </c>
-      <c r="G24">
-        <v>70.3</v>
-      </c>
-      <c r="H24" s="4">
-        <v>91.7</v>
-      </c>
-    </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B25" t="s">
-        <v>32</v>
-      </c>
-      <c r="C25" t="s">
-        <v>25</v>
-      </c>
-      <c r="D25">
-        <v>3.4</v>
-      </c>
-      <c r="E25">
-        <v>63.3</v>
-      </c>
-      <c r="F25">
-        <v>36.200000000000003</v>
-      </c>
-      <c r="G25" s="4">
-        <v>70.5</v>
-      </c>
-      <c r="H25">
-        <v>63.8</v>
-      </c>
-    </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C26" t="s">
         <v>25</v>
       </c>
       <c r="D26">
-        <v>57.9</v>
-      </c>
-      <c r="E26">
-        <v>50.4</v>
+        <v>93.4</v>
+      </c>
+      <c r="E26" s="4">
+        <v>95.8</v>
       </c>
       <c r="F26">
+        <v>58.4</v>
+      </c>
+      <c r="G26">
+        <v>81.599999999999994</v>
+      </c>
+      <c r="H26">
+        <v>29.2</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B27" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" t="s">
+        <v>25</v>
+      </c>
+      <c r="D27">
+        <v>33.799999999999997</v>
+      </c>
+      <c r="E27" s="4">
+        <v>93.3</v>
+      </c>
+      <c r="F27">
+        <v>64.900000000000006</v>
+      </c>
+      <c r="G27">
+        <v>63.2</v>
+      </c>
+      <c r="H27">
+        <v>7.1</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B28" t="s">
+        <v>36</v>
+      </c>
+      <c r="C28" t="s">
+        <v>25</v>
+      </c>
+      <c r="D28">
+        <v>15.6</v>
+      </c>
+      <c r="E28" s="4">
+        <v>77.599999999999994</v>
+      </c>
+      <c r="F28">
+        <v>24.3</v>
+      </c>
+      <c r="G28">
+        <v>5.3</v>
+      </c>
+      <c r="H28">
+        <v>53.5</v>
+      </c>
+    </row>
+    <row r="29" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B29" t="s">
+        <v>37</v>
+      </c>
+      <c r="C29" t="s">
+        <v>25</v>
+      </c>
+      <c r="D29">
+        <v>17.2</v>
+      </c>
+      <c r="E29">
+        <v>13.3</v>
+      </c>
+      <c r="F29" s="4">
+        <v>48.1</v>
+      </c>
+      <c r="G29">
+        <v>31.2</v>
+      </c>
+      <c r="H29">
+        <v>31.9</v>
+      </c>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B30" t="s">
+        <v>38</v>
+      </c>
+      <c r="C30" t="s">
+        <v>25</v>
+      </c>
+      <c r="D30">
         <v>5.0999999999999996</v>
       </c>
-      <c r="G26" s="4">
-        <v>63.4</v>
-      </c>
-      <c r="H26">
-        <v>4.8</v>
-      </c>
-    </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B27" t="s">
-        <v>34</v>
-      </c>
-      <c r="C27" t="s">
-        <v>25</v>
-      </c>
-      <c r="D27">
-        <v>93.4</v>
-      </c>
-      <c r="E27" s="4">
-        <v>95.8</v>
-      </c>
-      <c r="F27">
-        <v>58.4</v>
-      </c>
-      <c r="G27">
-        <v>81.599999999999994</v>
-      </c>
-      <c r="H27">
-        <v>29.2</v>
-      </c>
-    </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B28" t="s">
-        <v>35</v>
-      </c>
-      <c r="C28" t="s">
-        <v>25</v>
-      </c>
-      <c r="D28">
-        <v>33.799999999999997</v>
-      </c>
-      <c r="E28" s="4">
-        <v>93.3</v>
-      </c>
-      <c r="F28">
-        <v>64.900000000000006</v>
-      </c>
-      <c r="G28">
-        <v>63.2</v>
-      </c>
-      <c r="H28">
-        <v>7.1</v>
-      </c>
-    </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B29" t="s">
-        <v>36</v>
-      </c>
-      <c r="C29" t="s">
-        <v>25</v>
-      </c>
-      <c r="D29">
-        <v>15.6</v>
-      </c>
-      <c r="E29" s="4">
-        <v>77.599999999999994</v>
-      </c>
-      <c r="F29">
-        <v>24.3</v>
-      </c>
-      <c r="G29">
-        <v>5.3</v>
-      </c>
-      <c r="H29">
-        <v>53.5</v>
-      </c>
-    </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B30" t="s">
-        <v>37</v>
-      </c>
-      <c r="C30" t="s">
-        <v>25</v>
-      </c>
-      <c r="D30">
-        <v>17.2</v>
-      </c>
       <c r="E30">
-        <v>13.3</v>
-      </c>
-      <c r="F30" s="4">
-        <v>48.1</v>
-      </c>
-      <c r="G30">
-        <v>31.2</v>
+        <v>9.9</v>
+      </c>
+      <c r="F30">
+        <v>60.4</v>
+      </c>
+      <c r="G30" s="4">
+        <v>85.5</v>
       </c>
       <c r="H30">
-        <v>31.9</v>
-      </c>
-    </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B31" t="s">
-        <v>38</v>
-      </c>
-      <c r="C31" t="s">
-        <v>25</v>
-      </c>
-      <c r="D31">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="E31">
-        <v>9.9</v>
-      </c>
-      <c r="F31">
-        <v>60.4</v>
-      </c>
-      <c r="G31" s="4">
-        <v>85.5</v>
-      </c>
-      <c r="H31">
         <v>95.9</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B2:H31" xr:uid="{25C3A135-87E2-4A5E-8E06-586A6DE8385B}"/>
+  <autoFilter ref="B1:H30" xr:uid="{25C3A135-87E2-4A5E-8E06-586A6DE8385B}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4365,527 +4408,8 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A172548-7AE6-4D06-8BBB-21FD94D2FF8B}">
-  <dimension ref="B2:Q26"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="9.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.1796875" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="6" width="14.453125" customWidth="1"/>
-    <col min="7" max="7" width="17.1796875" customWidth="1"/>
-    <col min="8" max="8" width="13.36328125" customWidth="1"/>
-    <col min="12" max="12" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B2" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="F2" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="G2" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="H2" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="L2" t="s">
-        <v>39</v>
-      </c>
-      <c r="M2" t="s">
-        <v>41</v>
-      </c>
-      <c r="N2" t="s">
-        <v>40</v>
-      </c>
-      <c r="O2" s="12" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="3" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="4">
-        <v>98.5</v>
-      </c>
-      <c r="F3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H3" s="4">
-        <v>83.4</v>
-      </c>
-      <c r="K3" t="s">
-        <v>42</v>
-      </c>
-      <c r="L3">
-        <v>2</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-      <c r="N3">
-        <v>3</v>
-      </c>
-      <c r="O3" s="12">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="4">
-        <v>96.8</v>
-      </c>
-      <c r="F4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" t="s">
-        <v>8</v>
-      </c>
-      <c r="H4" s="4">
-        <v>84.7</v>
-      </c>
-      <c r="K4" t="s">
-        <v>43</v>
-      </c>
-      <c r="L4">
-        <v>2</v>
-      </c>
-      <c r="M4">
-        <v>2</v>
-      </c>
-      <c r="N4">
-        <v>2</v>
-      </c>
-      <c r="O4" s="12">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="4">
-        <v>76.7</v>
-      </c>
-      <c r="F5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" s="4">
-        <v>46</v>
-      </c>
-      <c r="K5" t="s">
-        <v>44</v>
-      </c>
-      <c r="L5">
-        <v>4</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
-      </c>
-      <c r="N5">
-        <v>3</v>
-      </c>
-      <c r="O5" s="12">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="4">
-        <v>83.9</v>
-      </c>
-      <c r="F6" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" t="s">
-        <v>19</v>
-      </c>
-      <c r="H6" s="4">
-        <v>60.3</v>
-      </c>
-      <c r="K6" t="s">
-        <v>45</v>
-      </c>
-      <c r="L6">
-        <v>2</v>
-      </c>
-      <c r="M6">
-        <v>1</v>
-      </c>
-      <c r="N6">
-        <v>1</v>
-      </c>
-      <c r="O6" s="12">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B7" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" s="4">
-        <v>70</v>
-      </c>
-      <c r="F7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G7" t="s">
-        <v>25</v>
-      </c>
-      <c r="H7" s="4">
-        <v>99</v>
-      </c>
-      <c r="K7" t="s">
-        <v>46</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
-        <v>0</v>
-      </c>
-      <c r="N7">
-        <v>5</v>
-      </c>
-      <c r="O7" s="12">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="4">
-        <v>57.9</v>
-      </c>
-      <c r="F8" t="s">
-        <v>34</v>
-      </c>
-      <c r="G8" t="s">
-        <v>25</v>
-      </c>
-      <c r="H8" s="4">
-        <v>95.8</v>
-      </c>
-      <c r="K8" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="L8" s="11">
-        <v>10</v>
-      </c>
-      <c r="M8" s="11">
-        <v>5</v>
-      </c>
-      <c r="N8" s="11">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="2:17" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B11" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="K11" t="s">
-        <v>49</v>
-      </c>
-      <c r="L11" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="M11" s="23"/>
-      <c r="N11" s="23"/>
-      <c r="O11" s="23"/>
-      <c r="P11" s="23"/>
-      <c r="Q11" s="23"/>
-    </row>
-    <row r="12" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B12" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" s="4">
-        <v>86</v>
-      </c>
-      <c r="F12" t="s">
-        <v>28</v>
-      </c>
-      <c r="G12" t="s">
-        <v>25</v>
-      </c>
-      <c r="H12" s="4">
-        <v>96.9</v>
-      </c>
-      <c r="K12" t="s">
-        <v>50</v>
-      </c>
-      <c r="L12" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="13" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B13" t="s">
-        <v>24</v>
-      </c>
-      <c r="C13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D13" s="4">
-        <v>74.900000000000006</v>
-      </c>
-      <c r="F13" t="s">
-        <v>21</v>
-      </c>
-      <c r="G13" t="s">
-        <v>19</v>
-      </c>
-      <c r="H13" s="4">
-        <v>43.9</v>
-      </c>
-      <c r="L13" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="14" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B14" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14" t="s">
-        <v>25</v>
-      </c>
-      <c r="D14" s="4">
-        <v>64.900000000000006</v>
-      </c>
-      <c r="F14" t="s">
-        <v>17</v>
-      </c>
-      <c r="G14" t="s">
-        <v>8</v>
-      </c>
-      <c r="H14" s="4">
-        <v>89.1</v>
-      </c>
-      <c r="L14" s="18" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="15" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B15" t="s">
-        <v>23</v>
-      </c>
-      <c r="C15" t="s">
-        <v>19</v>
-      </c>
-      <c r="D15" s="4">
-        <v>73.3</v>
-      </c>
-      <c r="F15" t="s">
-        <v>14</v>
-      </c>
-      <c r="G15" t="s">
-        <v>8</v>
-      </c>
-      <c r="H15" s="4">
-        <v>76.400000000000006</v>
-      </c>
-      <c r="L15" t="s">
-        <v>59</v>
-      </c>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
-      <c r="P15" s="1"/>
-      <c r="Q15" s="1"/>
-    </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.35">
-      <c r="B16" t="s">
-        <v>10</v>
-      </c>
-      <c r="C16" t="s">
-        <v>8</v>
-      </c>
-      <c r="D16" s="4">
-        <v>95.3</v>
-      </c>
-      <c r="K16" t="s">
-        <v>54</v>
-      </c>
-      <c r="L16" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B17" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" t="s">
-        <v>8</v>
-      </c>
-      <c r="D17" s="4">
-        <v>91</v>
-      </c>
-      <c r="K17" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="L17" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="M17" s="13"/>
-      <c r="N17" s="13"/>
-      <c r="O17" s="13"/>
-    </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B18" t="s">
-        <v>15</v>
-      </c>
-      <c r="C18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" s="4">
-        <v>87.1</v>
-      </c>
-    </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C19" t="s">
-        <v>8</v>
-      </c>
-      <c r="D19" s="4">
-        <v>54.9</v>
-      </c>
-    </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B21" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B22" t="s">
-        <v>38</v>
-      </c>
-      <c r="C22" t="s">
-        <v>25</v>
-      </c>
-      <c r="D22" s="4">
-        <v>95.9</v>
-      </c>
-    </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B23" t="s">
-        <v>31</v>
-      </c>
-      <c r="C23" t="s">
-        <v>25</v>
-      </c>
-      <c r="D23" s="4">
-        <v>91.7</v>
-      </c>
-    </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B24" t="s">
-        <v>32</v>
-      </c>
-      <c r="C24" t="s">
-        <v>25</v>
-      </c>
-      <c r="D24" s="4">
-        <v>63.8</v>
-      </c>
-    </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B25" t="s">
-        <v>36</v>
-      </c>
-      <c r="C25" t="s">
-        <v>25</v>
-      </c>
-      <c r="D25" s="4">
-        <v>53.5</v>
-      </c>
-    </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B26" t="s">
-        <v>37</v>
-      </c>
-      <c r="C26" t="s">
-        <v>25</v>
-      </c>
-      <c r="D26" s="4">
-        <v>31.9</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="L11:Q11"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86D0E5D6-7A76-4E6F-A0DD-59D4DB683A8B}">
-  <dimension ref="B2:T50"/>
+  <dimension ref="B2:T31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.6328125" customWidth="1"/>
@@ -5233,183 +4757,1381 @@
         <v>54.9</v>
       </c>
     </row>
-    <row r="35" spans="5:11" x14ac:dyDescent="0.35">
-      <c r="F35" t="s">
+    <row r="16" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="F16" t="s">
         <v>39</v>
       </c>
-      <c r="G35" t="s">
+      <c r="G16" t="s">
         <v>41</v>
       </c>
-      <c r="H35" t="s">
+      <c r="H16" t="s">
         <v>40</v>
       </c>
-      <c r="I35" s="12" t="s">
+      <c r="I16" s="12" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="36" spans="5:11" x14ac:dyDescent="0.35">
-      <c r="E36" t="s">
+    <row r="17" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="E17" t="s">
         <v>42</v>
       </c>
-      <c r="F36">
+      <c r="F17">
         <v>2</v>
       </c>
-      <c r="G36">
+      <c r="G17">
         <v>1</v>
       </c>
-      <c r="H36">
+      <c r="H17">
         <v>3</v>
       </c>
-      <c r="I36" s="12">
+      <c r="I17" s="12">
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="5:11" x14ac:dyDescent="0.35">
-      <c r="E37" t="s">
+    <row r="18" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="E18" t="s">
         <v>43</v>
       </c>
-      <c r="F37">
+      <c r="F18">
         <v>2</v>
       </c>
-      <c r="G37">
+      <c r="G18">
         <v>2</v>
       </c>
-      <c r="H37">
+      <c r="H18">
         <v>2</v>
       </c>
-      <c r="I37" s="12">
+      <c r="I18" s="12">
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="5:11" x14ac:dyDescent="0.35">
-      <c r="E38" t="s">
+    <row r="19" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="E19" t="s">
         <v>44</v>
       </c>
-      <c r="F38">
+      <c r="F19">
         <v>4</v>
       </c>
-      <c r="G38">
+      <c r="G19">
         <v>1</v>
       </c>
-      <c r="H38">
+      <c r="H19">
         <v>3</v>
       </c>
-      <c r="I38" s="12">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="39" spans="5:11" x14ac:dyDescent="0.35">
-      <c r="E39" t="s">
+      <c r="I19" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="E20" t="s">
         <v>45</v>
       </c>
-      <c r="F39">
+      <c r="F20">
         <v>2</v>
       </c>
-      <c r="G39">
+      <c r="G20">
         <v>1</v>
       </c>
-      <c r="H39">
+      <c r="H20">
         <v>1</v>
       </c>
-      <c r="I39" s="12">
+      <c r="I20" s="12">
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="5:11" x14ac:dyDescent="0.35">
-      <c r="E40" t="s">
+    <row r="21" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="E21" t="s">
         <v>46</v>
       </c>
-      <c r="F40">
+      <c r="F21">
         <v>0</v>
       </c>
-      <c r="G40">
+      <c r="G21">
         <v>0</v>
       </c>
-      <c r="H40">
+      <c r="H21">
         <v>5</v>
       </c>
-      <c r="I40" s="12">
+      <c r="I21" s="12">
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="5:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="E41" s="11" t="s">
+    <row r="22" spans="5:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="E22" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="F41" s="11">
+      <c r="F22" s="11">
         <v>10</v>
       </c>
-      <c r="G41" s="11">
+      <c r="G22" s="11">
         <v>5</v>
       </c>
-      <c r="H41" s="11">
+      <c r="H22" s="11">
         <v>14</v>
       </c>
     </row>
-    <row r="42" spans="5:11" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
-    <row r="44" spans="5:11" x14ac:dyDescent="0.35">
-      <c r="E44" t="s">
+    <row r="23" spans="5:13" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="25" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="E25" t="s">
         <v>49</v>
       </c>
-      <c r="F44" s="23" t="s">
+      <c r="F25" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="G44" s="23"/>
-      <c r="H44" s="23"/>
-      <c r="I44" s="23"/>
-      <c r="J44" s="23"/>
-      <c r="K44" s="23"/>
-    </row>
-    <row r="45" spans="5:11" x14ac:dyDescent="0.35">
-      <c r="E45" t="s">
+      <c r="G25" s="23"/>
+      <c r="H25" s="23"/>
+      <c r="I25" s="23"/>
+      <c r="J25" s="23"/>
+      <c r="K25" s="23"/>
+    </row>
+    <row r="26" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="E26" t="s">
         <v>50</v>
       </c>
-      <c r="F45" t="s">
+      <c r="F26" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="46" spans="5:11" x14ac:dyDescent="0.35">
-      <c r="F46" t="s">
+    <row r="27" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="F27" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="47" spans="5:11" x14ac:dyDescent="0.35">
-      <c r="F47" s="18" t="s">
+      <c r="M27">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="F28" s="18" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="48" spans="5:11" x14ac:dyDescent="0.35">
-      <c r="F48" t="s">
+    <row r="29" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="F29" t="s">
         <v>59</v>
       </c>
-      <c r="H48" s="1"/>
-      <c r="I48" s="1"/>
-      <c r="J48" s="1"/>
-      <c r="K48" s="1"/>
-    </row>
-    <row r="49" spans="5:9" x14ac:dyDescent="0.35">
-      <c r="E49" t="s">
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+    </row>
+    <row r="30" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="E30" t="s">
         <v>54</v>
       </c>
-      <c r="F49" t="s">
+      <c r="F30" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="50" spans="5:9" x14ac:dyDescent="0.35">
-      <c r="E50" s="13" t="s">
+    <row r="31" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="E31" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="F50" s="13" t="s">
+      <c r="F31" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="G50" s="13"/>
-      <c r="H50" s="13"/>
-      <c r="I50" s="13"/>
+      <c r="G31" s="13"/>
+      <c r="H31" s="13"/>
+      <c r="I31" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="F44:K44"/>
+    <mergeCell ref="F25:K25"/>
   </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA088233-5EF0-45F9-8BF7-5534FE391935}">
+  <dimension ref="B2:T73"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="4.6328125" customWidth="1"/>
+    <col min="2" max="2" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.36328125" customWidth="1"/>
+    <col min="6" max="6" width="14.453125" customWidth="1"/>
+    <col min="7" max="7" width="17.1796875" customWidth="1"/>
+    <col min="8" max="8" width="13.90625" customWidth="1"/>
+    <col min="9" max="9" width="4.6328125" customWidth="1"/>
+    <col min="11" max="11" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="4.453125" customWidth="1"/>
+    <col min="14" max="14" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="3.6328125" customWidth="1"/>
+    <col min="18" max="18" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B2" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B4" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="K4" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="L4" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="N4" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="O4" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="P4" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="R4" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="S4" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="T4" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="26">
+        <v>83.9</v>
+      </c>
+      <c r="F5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="26">
+        <v>99</v>
+      </c>
+      <c r="I5" s="1"/>
+      <c r="J5" t="s">
+        <v>27</v>
+      </c>
+      <c r="K5" t="s">
+        <v>25</v>
+      </c>
+      <c r="L5" s="26">
+        <v>86</v>
+      </c>
+      <c r="N5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O5" t="s">
+        <v>25</v>
+      </c>
+      <c r="P5" s="26">
+        <v>96.9</v>
+      </c>
+      <c r="R5" t="s">
+        <v>31</v>
+      </c>
+      <c r="S5" t="s">
+        <v>25</v>
+      </c>
+      <c r="T5" s="26">
+        <v>91.7</v>
+      </c>
+    </row>
+    <row r="6" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="26">
+        <v>70</v>
+      </c>
+      <c r="F6" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" s="28">
+        <v>95.8</v>
+      </c>
+      <c r="I6" s="1"/>
+      <c r="J6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L6" s="26">
+        <v>48.1</v>
+      </c>
+      <c r="N6" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="O6" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="P6" s="26">
+        <v>85.5</v>
+      </c>
+      <c r="R6" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="S6" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="T6" s="26">
+        <v>90.3</v>
+      </c>
+    </row>
+    <row r="7" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="26">
+        <v>76.7</v>
+      </c>
+      <c r="F7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="26">
+        <v>93.3</v>
+      </c>
+      <c r="I7" s="1"/>
+      <c r="J7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K7" t="s">
+        <v>19</v>
+      </c>
+      <c r="L7" s="26">
+        <v>73.3</v>
+      </c>
+      <c r="N7" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="O7" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="P7" s="26">
+        <v>84.3</v>
+      </c>
+      <c r="R7" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="S7" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="T7" s="28">
+        <v>84.7</v>
+      </c>
+    </row>
+    <row r="8" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="26">
+        <v>98.5</v>
+      </c>
+      <c r="F8" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="G8" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="26">
+        <v>77.599999999999994</v>
+      </c>
+      <c r="J8" t="s">
+        <v>10</v>
+      </c>
+      <c r="K8" t="s">
+        <v>8</v>
+      </c>
+      <c r="L8" s="26">
+        <v>95.3</v>
+      </c>
+      <c r="N8" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="O8" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="P8" s="26">
+        <v>70.5</v>
+      </c>
+      <c r="R8" s="33" t="s">
+        <v>22</v>
+      </c>
+      <c r="S8" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="T8" s="28">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="9" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="26">
+        <v>96.8</v>
+      </c>
+      <c r="F9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" t="s">
+        <v>8</v>
+      </c>
+      <c r="H9" s="26">
+        <v>84.7</v>
+      </c>
+      <c r="J9" t="s">
+        <v>9</v>
+      </c>
+      <c r="K9" t="s">
+        <v>8</v>
+      </c>
+      <c r="L9" s="26">
+        <v>91</v>
+      </c>
+      <c r="N9" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="O9" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="P9" s="26">
+        <v>63.4</v>
+      </c>
+      <c r="R9" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="S9" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="T9" s="26">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="J10" t="s">
+        <v>15</v>
+      </c>
+      <c r="K10" t="s">
+        <v>8</v>
+      </c>
+      <c r="L10" s="26">
+        <v>87.1</v>
+      </c>
+      <c r="N10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O10" t="s">
+        <v>8</v>
+      </c>
+      <c r="P10" s="26">
+        <v>89.1</v>
+      </c>
+      <c r="R10" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="S10" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="T10" s="26">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="F11" s="24"/>
+      <c r="G11" s="24"/>
+      <c r="J11" s="24"/>
+      <c r="K11" s="24"/>
+      <c r="L11" s="24"/>
+      <c r="N11" t="s">
+        <v>14</v>
+      </c>
+      <c r="O11" t="s">
+        <v>8</v>
+      </c>
+      <c r="P11" s="26">
+        <v>76.400000000000006</v>
+      </c>
+      <c r="R11" s="24"/>
+      <c r="S11" s="24"/>
+    </row>
+    <row r="12" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
+      <c r="J12" s="24"/>
+      <c r="K12" s="24"/>
+      <c r="L12" s="24"/>
+      <c r="P12" s="29"/>
+      <c r="R12" s="24"/>
+      <c r="S12" s="24"/>
+    </row>
+    <row r="13" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="15" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B15" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="J15" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="K15" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="L15" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="N15" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="O15" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="P15" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="R15" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="S15" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="T15" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" t="s">
+        <v>25</v>
+      </c>
+      <c r="D16" s="29">
+        <v>83.9</v>
+      </c>
+      <c r="F16" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" t="s">
+        <v>25</v>
+      </c>
+      <c r="H16" s="29">
+        <v>99</v>
+      </c>
+      <c r="I16" s="1"/>
+      <c r="J16" t="s">
+        <v>27</v>
+      </c>
+      <c r="K16" t="s">
+        <v>25</v>
+      </c>
+      <c r="L16" s="29">
+        <v>86</v>
+      </c>
+      <c r="M16" s="30"/>
+      <c r="N16" t="s">
+        <v>28</v>
+      </c>
+      <c r="O16" t="s">
+        <v>25</v>
+      </c>
+      <c r="P16" s="29">
+        <v>96.9</v>
+      </c>
+      <c r="R16" t="s">
+        <v>31</v>
+      </c>
+      <c r="S16" t="s">
+        <v>25</v>
+      </c>
+      <c r="T16" s="29">
+        <v>91.7</v>
+      </c>
+    </row>
+    <row r="17" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17" s="29">
+        <v>70</v>
+      </c>
+      <c r="F17" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="G17" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="H17" s="32">
+        <v>95.8</v>
+      </c>
+      <c r="I17" s="1"/>
+      <c r="J17" t="s">
+        <v>37</v>
+      </c>
+      <c r="K17" t="s">
+        <v>25</v>
+      </c>
+      <c r="L17" s="29">
+        <v>48.1</v>
+      </c>
+      <c r="M17" s="30"/>
+      <c r="N17" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="O17" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="P17" s="31">
+        <v>85.5</v>
+      </c>
+      <c r="R17" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="S17" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="T17" s="31">
+        <v>90.3</v>
+      </c>
+    </row>
+    <row r="18" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B18" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" t="s">
+        <v>19</v>
+      </c>
+      <c r="D18" s="29">
+        <v>76.7</v>
+      </c>
+      <c r="F18" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="G18" t="s">
+        <v>25</v>
+      </c>
+      <c r="H18" s="29">
+        <v>93.3</v>
+      </c>
+      <c r="I18" s="1"/>
+      <c r="J18" t="s">
+        <v>23</v>
+      </c>
+      <c r="K18" t="s">
+        <v>19</v>
+      </c>
+      <c r="L18" s="29">
+        <v>73.3</v>
+      </c>
+      <c r="M18" s="30"/>
+      <c r="N18" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="O18" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="P18" s="31">
+        <v>84.3</v>
+      </c>
+      <c r="R18" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="S18" s="34" t="s">
+        <v>19</v>
+      </c>
+      <c r="T18" s="35">
+        <v>84.7</v>
+      </c>
+    </row>
+    <row r="19" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" s="29">
+        <v>98.5</v>
+      </c>
+      <c r="F19" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H19" s="31">
+        <v>77.599999999999994</v>
+      </c>
+      <c r="J19" t="s">
+        <v>10</v>
+      </c>
+      <c r="K19" t="s">
+        <v>8</v>
+      </c>
+      <c r="L19" s="29">
+        <v>95.3</v>
+      </c>
+      <c r="M19" s="30"/>
+      <c r="N19" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="O19" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="P19" s="31">
+        <v>70.5</v>
+      </c>
+      <c r="R19" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="S19" s="34" t="s">
+        <v>19</v>
+      </c>
+      <c r="T19" s="35">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="20" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B20" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="29">
+        <v>96.8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" t="s">
+        <v>8</v>
+      </c>
+      <c r="H20" s="29">
+        <v>84.7</v>
+      </c>
+      <c r="J20" t="s">
+        <v>9</v>
+      </c>
+      <c r="K20" t="s">
+        <v>8</v>
+      </c>
+      <c r="L20" s="29">
+        <v>91</v>
+      </c>
+      <c r="M20" s="30"/>
+      <c r="N20" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O20" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="P20" s="31">
+        <v>63.4</v>
+      </c>
+      <c r="R20" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="S20" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="T20" s="31">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="21" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B21" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="C21" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="D21" s="24"/>
+      <c r="F21" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="G21" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="H21" s="24"/>
+      <c r="J21" t="s">
+        <v>15</v>
+      </c>
+      <c r="K21" t="s">
+        <v>8</v>
+      </c>
+      <c r="L21" s="29">
+        <v>87.1</v>
+      </c>
+      <c r="N21" t="s">
+        <v>17</v>
+      </c>
+      <c r="O21" t="s">
+        <v>8</v>
+      </c>
+      <c r="P21" s="29">
+        <v>89.1</v>
+      </c>
+      <c r="R21" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="S21" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="T21" s="31">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="F22" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="G22" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="J22" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="K22" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="L22" s="24"/>
+      <c r="N22" t="s">
+        <v>14</v>
+      </c>
+      <c r="O22" t="s">
+        <v>8</v>
+      </c>
+      <c r="P22" s="29">
+        <v>76.400000000000006</v>
+      </c>
+      <c r="R22" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="S22" s="25" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="F23" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="G23" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="J23" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="K23" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="L23" s="24"/>
+      <c r="N23" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="O23" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="P23" s="24"/>
+      <c r="R23" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="S23" s="25" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="J24" s="24"/>
+      <c r="K24" s="24"/>
+      <c r="L24" s="24"/>
+      <c r="P24" s="24"/>
+      <c r="R24" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="S24" s="25" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="J25" s="24"/>
+      <c r="K25" s="24"/>
+      <c r="L25" s="24"/>
+      <c r="P25" s="24"/>
+      <c r="R25" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="S25" s="25" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="J26" s="24"/>
+      <c r="K26" s="24"/>
+      <c r="L26" s="24"/>
+      <c r="P26" s="24"/>
+      <c r="R26" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="S26" s="25" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B27" s="1"/>
+      <c r="F27" s="37"/>
+      <c r="J27" s="24"/>
+      <c r="K27" s="24"/>
+      <c r="L27" s="24"/>
+      <c r="P27" s="24"/>
+    </row>
+    <row r="28" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="J28" s="24"/>
+      <c r="K28" s="24"/>
+      <c r="L28" s="24"/>
+      <c r="P28" s="24"/>
+    </row>
+    <row r="29" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="J29" s="24"/>
+      <c r="K29" s="24"/>
+      <c r="L29" s="24"/>
+      <c r="P29" s="24"/>
+    </row>
+    <row r="30" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B30" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="E30" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F30" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="G30" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="H30" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="J30" s="24"/>
+      <c r="K30" s="24"/>
+      <c r="L30" s="24"/>
+      <c r="P30" s="24"/>
+    </row>
+    <row r="31" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B31" t="s">
+        <v>36</v>
+      </c>
+      <c r="C31" t="s">
+        <v>25</v>
+      </c>
+      <c r="D31">
+        <v>15.6</v>
+      </c>
+      <c r="E31" s="4">
+        <v>77.599999999999994</v>
+      </c>
+      <c r="F31">
+        <v>24.3</v>
+      </c>
+      <c r="G31">
+        <v>5.3</v>
+      </c>
+      <c r="H31">
+        <v>53.5</v>
+      </c>
+      <c r="J31" s="24"/>
+      <c r="K31" s="24"/>
+      <c r="L31" s="24"/>
+      <c r="P31" s="24"/>
+    </row>
+    <row r="32" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="J32" s="24"/>
+      <c r="K32" s="24"/>
+      <c r="L32" s="24"/>
+      <c r="P32" s="24"/>
+    </row>
+    <row r="33" spans="10:16" x14ac:dyDescent="0.35">
+      <c r="J33" s="24"/>
+      <c r="K33" s="24"/>
+      <c r="L33" s="24"/>
+      <c r="P33" s="24"/>
+    </row>
+    <row r="34" spans="10:16" x14ac:dyDescent="0.35">
+      <c r="J34" s="24"/>
+      <c r="K34" s="24"/>
+      <c r="L34" s="24"/>
+      <c r="P34" s="24"/>
+    </row>
+    <row r="35" spans="10:16" x14ac:dyDescent="0.35">
+      <c r="J35" s="24"/>
+      <c r="K35" s="24"/>
+      <c r="L35" s="24"/>
+      <c r="P35" s="24"/>
+    </row>
+    <row r="36" spans="10:16" x14ac:dyDescent="0.35">
+      <c r="J36" s="24"/>
+      <c r="K36" s="24"/>
+      <c r="L36" s="24"/>
+      <c r="P36" s="24"/>
+    </row>
+    <row r="37" spans="10:16" x14ac:dyDescent="0.35">
+      <c r="J37" s="24"/>
+      <c r="K37" s="24"/>
+      <c r="L37" s="24"/>
+      <c r="P37" s="24"/>
+    </row>
+    <row r="38" spans="10:16" x14ac:dyDescent="0.35">
+      <c r="J38" s="24"/>
+      <c r="K38" s="24"/>
+      <c r="L38" s="24"/>
+      <c r="P38" s="24"/>
+    </row>
+    <row r="39" spans="10:16" x14ac:dyDescent="0.35">
+      <c r="J39" s="24"/>
+      <c r="K39" s="24"/>
+      <c r="L39" s="24"/>
+      <c r="P39" s="24"/>
+    </row>
+    <row r="40" spans="10:16" x14ac:dyDescent="0.35">
+      <c r="J40" s="24"/>
+      <c r="K40" s="24"/>
+      <c r="L40" s="24"/>
+      <c r="P40" s="24"/>
+    </row>
+    <row r="41" spans="10:16" x14ac:dyDescent="0.35">
+      <c r="J41" s="24"/>
+      <c r="K41" s="24"/>
+      <c r="L41" s="24"/>
+      <c r="P41" s="24"/>
+    </row>
+    <row r="42" spans="10:16" x14ac:dyDescent="0.35">
+      <c r="J42" s="24"/>
+      <c r="K42" s="24"/>
+      <c r="L42" s="24"/>
+      <c r="P42" s="24"/>
+    </row>
+    <row r="43" spans="10:16" x14ac:dyDescent="0.35">
+      <c r="J43" s="24"/>
+      <c r="K43" s="24"/>
+      <c r="L43" s="24"/>
+      <c r="P43" s="24"/>
+    </row>
+    <row r="44" spans="10:16" x14ac:dyDescent="0.35">
+      <c r="J44" s="24"/>
+      <c r="K44" s="24"/>
+      <c r="L44" s="24"/>
+      <c r="P44" s="24"/>
+    </row>
+    <row r="45" spans="10:16" x14ac:dyDescent="0.35">
+      <c r="J45" s="24"/>
+      <c r="K45" s="24"/>
+      <c r="L45" s="24"/>
+      <c r="P45" s="24"/>
+    </row>
+    <row r="46" spans="10:16" x14ac:dyDescent="0.35">
+      <c r="J46" s="24"/>
+      <c r="K46" s="24"/>
+      <c r="L46" s="24"/>
+      <c r="P46" s="24"/>
+    </row>
+    <row r="47" spans="10:16" x14ac:dyDescent="0.35">
+      <c r="J47" s="24"/>
+      <c r="K47" s="24"/>
+      <c r="L47" s="24"/>
+      <c r="P47" s="24"/>
+    </row>
+    <row r="48" spans="10:16" x14ac:dyDescent="0.35">
+      <c r="J48" s="24"/>
+      <c r="K48" s="24"/>
+      <c r="L48" s="24"/>
+      <c r="P48" s="24"/>
+    </row>
+    <row r="49" spans="6:16" x14ac:dyDescent="0.35">
+      <c r="J49" s="24"/>
+      <c r="K49" s="24"/>
+      <c r="L49" s="24"/>
+      <c r="P49" s="24"/>
+    </row>
+    <row r="50" spans="6:16" x14ac:dyDescent="0.35">
+      <c r="G50" t="s">
+        <v>39</v>
+      </c>
+      <c r="H50" t="s">
+        <v>41</v>
+      </c>
+      <c r="I50" t="s">
+        <v>40</v>
+      </c>
+      <c r="J50" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="K50" s="24"/>
+      <c r="L50" s="24"/>
+      <c r="P50" s="24"/>
+    </row>
+    <row r="51" spans="6:16" x14ac:dyDescent="0.35">
+      <c r="F51" t="s">
+        <v>42</v>
+      </c>
+      <c r="G51">
+        <v>2</v>
+      </c>
+      <c r="H51">
+        <v>1</v>
+      </c>
+      <c r="I51" s="25">
+        <v>3</v>
+      </c>
+      <c r="J51" s="12">
+        <v>6</v>
+      </c>
+      <c r="K51" s="24"/>
+      <c r="L51" s="24"/>
+      <c r="P51" s="24"/>
+    </row>
+    <row r="52" spans="6:16" x14ac:dyDescent="0.35">
+      <c r="F52" t="s">
+        <v>43</v>
+      </c>
+      <c r="G52">
+        <v>2</v>
+      </c>
+      <c r="H52" s="25">
+        <v>2</v>
+      </c>
+      <c r="I52" s="25">
+        <v>2</v>
+      </c>
+      <c r="J52" s="12">
+        <v>6</v>
+      </c>
+      <c r="K52" s="24"/>
+      <c r="L52" s="24"/>
+    </row>
+    <row r="53" spans="6:16" x14ac:dyDescent="0.35">
+      <c r="F53" t="s">
+        <v>44</v>
+      </c>
+      <c r="G53" s="25">
+        <v>4</v>
+      </c>
+      <c r="H53">
+        <v>1</v>
+      </c>
+      <c r="I53" s="25">
+        <v>3</v>
+      </c>
+      <c r="J53" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="54" spans="6:16" x14ac:dyDescent="0.35">
+      <c r="F54" t="s">
+        <v>45</v>
+      </c>
+      <c r="G54">
+        <v>2</v>
+      </c>
+      <c r="H54">
+        <v>1</v>
+      </c>
+      <c r="I54">
+        <v>1</v>
+      </c>
+      <c r="J54" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55" spans="6:16" x14ac:dyDescent="0.35">
+      <c r="F55" t="s">
+        <v>46</v>
+      </c>
+      <c r="G55">
+        <v>0</v>
+      </c>
+      <c r="H55">
+        <v>0</v>
+      </c>
+      <c r="I55">
+        <v>5</v>
+      </c>
+      <c r="J55" s="12">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="56" spans="6:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="F56" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="G56" s="11">
+        <v>10</v>
+      </c>
+      <c r="H56" s="11">
+        <v>5</v>
+      </c>
+      <c r="I56" s="11">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="57" spans="6:16" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="67" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="E67" t="s">
+        <v>49</v>
+      </c>
+      <c r="F67" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="G67" s="23"/>
+      <c r="H67" s="23"/>
+      <c r="I67" s="23"/>
+      <c r="J67" s="23"/>
+      <c r="K67" s="23"/>
+    </row>
+    <row r="68" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="E68" t="s">
+        <v>50</v>
+      </c>
+      <c r="F68" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="69" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="F69" t="s">
+        <v>52</v>
+      </c>
+      <c r="M69">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="F70" s="18" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="71" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="F71" t="s">
+        <v>59</v>
+      </c>
+      <c r="H71" s="1"/>
+      <c r="I71" s="1"/>
+      <c r="J71" s="1"/>
+      <c r="K71" s="1"/>
+    </row>
+    <row r="72" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="E72" t="s">
+        <v>54</v>
+      </c>
+      <c r="F72" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="73" spans="5:13" x14ac:dyDescent="0.35">
+      <c r="E73" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="F73" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="G73" s="13"/>
+      <c r="H73" s="13"/>
+      <c r="I73" s="13"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="F67:K67"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="F18" location="'Stage 1'!A1" display="VP6" xr:uid="{11E86EC5-B611-4BFA-BA48-BEFD10AC62C8}"/>
+    <hyperlink ref="F19" location="'Stage 1'!A1" display="VP7" xr:uid="{CC8CB78E-623A-44BF-98AC-AF14F818CE53}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update Flowchart ML development.xksx
</commit_message>
<xml_diff>
--- a/1.training_model/supplementary/Data Tabulation - Flowchart.xlsx
+++ b/1.training_model/supplementary/Data Tabulation - Flowchart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sitisyaziyah\source\repos\DeviceCluster\1.training_model\supplementary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{971519B7-5377-4244-AFDD-99390543FF09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C177ABD-7CF8-4571-93F1-94E5AF7E7F48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="717" firstSheet="2" activeTab="9" xr2:uid="{E471D6E3-533D-4285-ABDC-6FF3DFDEE99D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="717" firstSheet="3" activeTab="10" xr2:uid="{E471D6E3-533D-4285-ABDC-6FF3DFDEE99D}"/>
   </bookViews>
   <sheets>
     <sheet name="Obs-flowchart" sheetId="19" state="hidden" r:id="rId1"/>
@@ -23,7 +23,8 @@
     <sheet name="Stage 2" sheetId="6" r:id="rId8"/>
     <sheet name="Stage 3" sheetId="7" r:id="rId9"/>
     <sheet name="Stage 4" sheetId="13" r:id="rId10"/>
-    <sheet name="transpose" sheetId="3" state="hidden" r:id="rId11"/>
+    <sheet name="try and error" sheetId="24" r:id="rId11"/>
+    <sheet name="transpose" sheetId="3" state="hidden" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Draft Data'!#REF!</definedName>
@@ -31,7 +32,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Stage 2'!$B$2:$H$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Stage 3'!$B$2:$H$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Stage 4'!#REF!</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">transpose!$B$3:$AE$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">transpose!$B$3:$AE$12</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -11965,6 +11966,72 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>177800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>501650</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>157875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CFB743D4-5788-2011-A2EC-588B2A2894CA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="3124200" y="361950"/>
+          <a:ext cx="5911850" cy="3294775"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -12825,6 +12892,16 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4779006-2C51-4123-8965-52E24C209B6E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24775ADE-03D3-4D0A-807B-37E1A793A03E}">
   <dimension ref="B3:AE12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>